<commit_message>
Update: Replace with formatted OEE table
</commit_message>
<xml_diff>
--- a/OEE_Audit_Report_Production_Line_A.xlsx
+++ b/OEE_Audit_Report_Production_Line_A.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\batiz\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4EE19A-AEC2-4EF5-AD73-29FED2771E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A71C6C-2667-40B6-88E9-F1FB20988574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Configuración de Excel para OEE" sheetId="1" r:id="rId1"/>
+    <sheet name="OEE_Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Concept</t>
   </si>
@@ -81,42 +81,58 @@
   </si>
   <si>
     <t>Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri Light"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri Light"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri Light"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri Light"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -142,7 +158,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -154,12 +170,120 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -176,60 +300,134 @@
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2F0F3F49-19D9-425B-B733-8264EBBA8A19}" name="OEE_Metrics" displayName="OEE_Metrics" ref="A1:E6" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:E6" xr:uid="{2F0F3F49-19D9-425B-B733-8264EBBA8A19}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{EC6C963B-EEB0-43B7-994A-46E50E8EBCFA}" name="Concept" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{A986C3D7-3B0B-4622-B016-F592C94363FA}" name="Value" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{73AC4D8B-1898-4695-BC66-ED9ABC5F5795}" name="Unit" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{E03A14BC-A2CC-4BA4-97B9-EEF8A54BA412}" name="Metric" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{9E645F7B-E6F7-49AF-94AA-DA36E7F59D5E}" name="Value " dataDxfId="1" dataCellStyle="Porcentaje"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Metropolitano">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Metropolitano">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="162F33"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="EAF0E0"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285F4"/>
+        <a:srgbClr val="50B4C8"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EA4335"/>
+        <a:srgbClr val="A8B97F"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="FBBC04"/>
+        <a:srgbClr val="9B9256"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34A853"/>
+        <a:srgbClr val="657689"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="FF6D01"/>
+        <a:srgbClr val="7A855D"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46BDC6"/>
+        <a:srgbClr val="84AC9D"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="2370CD"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="877589"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Metropolitano">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Metropolitano">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -238,76 +436,73 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="70000"/>
+                <a:satMod val="100000"/>
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="75000"/>
+                <a:satMod val="101000"/>
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="82000"/>
+                <a:satMod val="104000"/>
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="2700000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
+                <a:tint val="97000"/>
+                <a:satMod val="100000"/>
                 <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="100000"/>
                 <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="80000"/>
+                <a:satMod val="100000"/>
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="2700000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -337,38 +532,22 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Metropolitan" id="{4C5440D6-04D2-4954-96CF-F251137069B2}" vid="{79CFCA13-9412-4290-BB4B-85112F88857B}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
@@ -394,8 +573,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="8" t="s">
         <v>15</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
@@ -483,5 +665,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>